<commit_message>
docs: completar analisis fuentes capturas y guia de exposicion
</commit_message>
<xml_diff>
--- a/Semana09/outputs/semana09/Boleta_Grupo_B.xlsx
+++ b/Semana09/outputs/semana09/Boleta_Grupo_B.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parámetros" sheetId="1" r:id="R6a348850fd4943ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boleta" sheetId="2" r:id="R5dae76dbc8774de6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos" sheetId="3" r:id="R3500b38a67924075"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Explicación" sheetId="4" r:id="R999c3f5d7ea1423c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parámetros" sheetId="1" r:id="R2c6dbf4bb9fa4855"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boleta" sheetId="2" r:id="R3873d9ad6481442a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos" sheetId="3" r:id="Rd84bb014470d4ac1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Explicación" sheetId="4" r:id="R2850336088594e7d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -372,13 +372,13 @@
         <x:v>1230</x:v>
       </x:c>
       <x:c r="C4" s="5" t="str">
-        <x:v>Actividad Grupo B; supuesto académico</x:v>
+        <x:v>D.S. 015-2026-TR, art. 1.2; desde 01/10/2026</x:v>
       </x:c>
       <x:c r="D4" s="5" t="str">
         <x:v>26/10/2026</x:v>
       </x:c>
       <x:c r="E4" s="5" t="str">
-        <x:v>Actividad_Grupo_B.docx, sección 4</x:v>
+        <x:v>https://busquedas.elperuano.pe/dispositivo/EX/2559163-1</x:v>
       </x:c>
       <x:c r="F4" s="1"/>
       <x:c r="G4" s="1"/>
@@ -762,19 +762,19 @@
     </x:row>
     <x:row r="28" ht="64" customHeight="1">
       <x:c r="A28" s="1" t="str">
-        <x:v>RMV oficial</x:v>
+        <x:v>Vigencia RMV</x:v>
       </x:c>
       <x:c r="B28" s="1" t="str">
-        <x:v>Por verificar</x:v>
+        <x:v>01/10/2026</x:v>
       </x:c>
       <x:c r="C28" s="5" t="str">
-        <x:v>No se afirma vigencia legal a partir del enunciado.</x:v>
+        <x:v>S/ 1,230 según art. 1.2 del D.S. 015-2026-TR.</x:v>
       </x:c>
       <x:c r="D28" s="5" t="str">
         <x:v>26/10/2026</x:v>
       </x:c>
       <x:c r="E28" s="5" t="str">
-        <x:v>https://www.gob.pe/mtpe</x:v>
+        <x:v>https://busquedas.elperuano.pe/dispositivo/EX/2559163-1</x:v>
       </x:c>
       <x:c r="F28" s="1"/>
       <x:c r="G28" s="1"/>

</xml_diff>